<commit_message>
Improve clock config around STM32F4 family
</commit_message>
<xml_diff>
--- a/Info/STM32any CPU Frequency chart.xlsx
+++ b/Info/STM32any CPU Frequency chart.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="78">
   <si>
     <t xml:space="preserve">Max frequency</t>
   </si>
@@ -142,6 +142,9 @@
     <t xml:space="preserve">50 MHz</t>
   </si>
   <si>
+    <t xml:space="preserve">STM32F411</t>
+  </si>
+  <si>
     <t xml:space="preserve">STM32F412</t>
   </si>
   <si>
@@ -154,37 +157,37 @@
     <t xml:space="preserve">STM32F417</t>
   </si>
   <si>
+    <t xml:space="preserve">STM32F423</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM32F427</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180 MHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45 MHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90 MHz</t>
+  </si>
+  <si>
     <t xml:space="preserve">STM32F429</t>
   </si>
   <si>
+    <t xml:space="preserve">STM32F437</t>
+  </si>
+  <si>
     <t xml:space="preserve">STM32F439</t>
   </si>
   <si>
     <t xml:space="preserve">STM32F446</t>
   </si>
   <si>
-    <t xml:space="preserve">180 MHz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">90 MHz</t>
-  </si>
-  <si>
     <t xml:space="preserve">STM32F469</t>
   </si>
   <si>
     <t xml:space="preserve">STM32F479</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM32F40xx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM32F41xx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM32F427xx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM32F437xx</t>
   </si>
   <si>
     <t xml:space="preserve">STM32F7 Series</t>
@@ -265,6 +268,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -286,6 +290,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -330,16 +335,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -466,760 +475,757 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2"/>
-      <c r="C19" s="1" t="s">
+      <c r="B19" s="3"/>
+      <c r="C19" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="2"/>
+      <c r="D19" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="B21" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="B23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="B24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="B25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C36" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D36" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="B36" s="2" t="s">
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C37" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D37" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="B37" s="2" t="s">
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C40" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D40" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="2" t="s">
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C42" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D42" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B39" s="2" t="s">
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C43" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="D43" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="C44" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B40" s="2" t="s">
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C45" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>32</v>
+      <c r="D45" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C48" s="1" t="s">
-        <v>55</v>
+      <c r="C47" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>57</v>
+      <c r="A50" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
+      <c r="A51" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>57</v>
+      <c r="D51" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>57</v>
+      <c r="A52" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>57</v>
+      <c r="A53" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>57</v>
+      <c r="A54" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>57</v>
+      <c r="A55" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>57</v>
+      <c r="A56" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C60" s="1" t="s">
+      <c r="A57" s="1" t="s">
         <v>67</v>
       </c>
+      <c r="B57" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C59" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F61" s="3"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F62" s="2"/>
+      <c r="A62" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
+      <c r="A63" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>70</v>
+      <c r="D63" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>70</v>
-      </c>
+      <c r="A64" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F64" s="3"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F65" s="2"/>
+      <c r="A65" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F66" s="2"/>
+      <c r="A66" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>70</v>
+      <c r="A67" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>